<commit_message>
Replace internal attribution labels with external-facing wording
The workbook carried 36 'per HJ' notes and 3 'Added by Claude' cells.
Both were internal working shorthand: HJ identified the client by name
from the session profile, and 'Added by Claude' named the tool. Neither
belongs in a document going to a bank.

  per HJ            -> per management
  Added by Claude   -> Not in original brief

The audit trail is preserved - it still distinguishes figures supplied by
management from lines added during modelling - but reads as a normal
finance document. Product references to Claude on the AI Subscriptions
tab are left alone; those are genuine tool names.

No figures changed: CAPEX 121,158; Year-1 OPEX 691,253; peak cash deficit
76,726; funding required 237,461; headroom (37,461).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016f46jvoRwWpeUbBhAUhLud
</commit_message>
<xml_diff>
--- a/orizuru/Orizuru_CAPEX_OPEX_Model.xlsx
+++ b/orizuru/Orizuru_CAPEX_OPEX_Model.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Funding Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Assumptions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="CAPEX Summary" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="CAPEX Detail" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Unit Setup (1 Unit)" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="OPEX Summary" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="OPEX Monthly" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Marketing Comparison" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="AI Subscriptions" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAPEX Summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAPEX Detail" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Setup (1 Unit)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OPEX Summary" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OPEX Monthly" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marketing Comparison" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Subscriptions" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="B35" s="9" t="inlineStr">
         <is>
-          <t>Key lever, or a figure you supplied.</t>
+          <t>Key lever, or a figure supplied by management.</t>
         </is>
       </c>
     </row>
@@ -1312,7 +1312,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>HJ item 5. Feeds the 'AI subscriptions' line in the OPEX model. USD converted at the pegged AED rate.</t>
+          <t>Specified by management. Feeds the 'AI subscriptions' line in the OPEX model. USD converted at the pegged AED rate.</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2260,7 +2260,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>All figures AED unless stated. Blue = editable input. Yellow = figure supplied by HJ or a key lever.</t>
+          <t>All figures AED unless stated. Blue = editable input. Yellow = figure supplied by management or a key lever.</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2321,7 +2321,7 @@
       </c>
       <c r="C6" s="36" t="inlineStr">
         <is>
-          <t>Both options run in Months 1–2 per HJ. From Month 3 the model keeps whichever you select here. Select 'Both' to keep running them in parallel all year.</t>
+          <t>Both options run in Months 1–2 per management. From Month 3 the model keeps whichever you select here. Select 'Both' to keep running them in parallel all year.</t>
         </is>
       </c>
       <c r="J6" s="37" t="inlineStr">
@@ -2341,7 +2341,7 @@
       </c>
       <c r="C7" s="36" t="inlineStr">
         <is>
-          <t>Per HJ: run both marketing options together for the first 2 months to see which works.</t>
+          <t>Per management: run both marketing options together for the first 2 months to see which works.</t>
         </is>
       </c>
     </row>
@@ -2620,7 +2620,7 @@
       </c>
       <c r="G18" s="21" t="inlineStr">
         <is>
-          <t>Per HJ: directors will NOT draw a salary. Note for the bank — this understates the true cost of running the business, since two directors are working unpaid.</t>
+          <t>Per management: directors will NOT draw a salary. Note for the bank — this understates the true cost of running the business, since two directors are working unpaid.</t>
         </is>
       </c>
     </row>
@@ -2650,7 +2650,7 @@
       </c>
       <c r="G19" s="21" t="inlineStr">
         <is>
-          <t>Per HJ: 1 person.</t>
+          <t>Per management: 1 person.</t>
         </is>
       </c>
     </row>
@@ -2680,7 +2680,7 @@
       </c>
       <c r="G20" s="21" t="inlineStr">
         <is>
-          <t>Per HJ: AED 3,000/month.</t>
+          <t>Per management: AED 3,000/month.</t>
         </is>
       </c>
     </row>
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G25" s="21" t="inlineStr">
         <is>
-          <t>Per HJ: 2–4 persons.</t>
+          <t>Per management: 2–4 persons.</t>
         </is>
       </c>
     </row>
@@ -2843,7 +2843,7 @@
       </c>
       <c r="G26" s="21" t="inlineStr">
         <is>
-          <t>Per HJ: AED 500–700 per person.</t>
+          <t>Per management: AED 500–700 per person.</t>
         </is>
       </c>
     </row>
@@ -2976,7 +2976,7 @@
       </c>
       <c r="G31" s="21" t="inlineStr">
         <is>
-          <t>Per HJ: 4–6 persons.</t>
+          <t>Per management: 4–6 persons.</t>
         </is>
       </c>
     </row>
@@ -3006,7 +3006,7 @@
       </c>
       <c r="G32" s="21" t="inlineStr">
         <is>
-          <t>Per HJ: AED 180–300 per person.</t>
+          <t>Per management: AED 180–300 per person.</t>
         </is>
       </c>
     </row>
@@ -3036,7 +3036,7 @@
       </c>
       <c r="G33" s="21" t="inlineStr">
         <is>
-          <t>Per HJ: AED 1,350–1,500.</t>
+          <t>Per management: AED 1,350–1,500.</t>
         </is>
       </c>
     </row>
@@ -3066,7 +3066,7 @@
       </c>
       <c r="G34" s="21" t="inlineStr">
         <is>
-          <t>Not in HJ's original list but unavoidable — a physical room needs connectivity and machines.</t>
+          <t>Not in the original brief but unavoidable — a physical room needs connectivity and machines.</t>
         </is>
       </c>
     </row>
@@ -3096,7 +3096,7 @@
       </c>
       <c r="G35" s="21" t="inlineStr">
         <is>
-          <t>Not in HJ's original list. 4–6 people in a physical room with no supervisor will drift. Recommend keeping this.</t>
+          <t>Not in the original brief. 4–6 people in a physical room with no supervisor will drift. Recommend keeping this.</t>
         </is>
       </c>
     </row>
@@ -3156,14 +3156,14 @@
       </c>
       <c r="G37" s="21" t="inlineStr">
         <is>
-          <t>Not in HJ's original list. Engaging staff outside the UAE needs a compliant contracting route. Flagging it rather than pretending it is free.</t>
+          <t>Not in the original brief. Engaging staff outside the UAE needs a compliant contracting route. Flagging it rather than pretending it is free.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>5.  UNIT-ACQUISITION COMMISSION  —  the 2% per HJ</t>
+          <t>5.  UNIT-ACQUISITION COMMISSION  —  the 2% per management</t>
         </is>
       </c>
       <c r="B38" s="5" t="n"/>
@@ -3199,7 +3199,7 @@
       </c>
       <c r="G39" s="21" t="inlineStr">
         <is>
-          <t>Per HJ: 2% for each unit signed, ONGOING on that unit's monthly revenue.</t>
+          <t>Per management: 2% for each unit signed, ONGOING on that unit's monthly revenue.</t>
         </is>
       </c>
     </row>
@@ -3336,7 +3336,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="22" customHeight="1">
+    <row r="45" ht="33" customHeight="1">
       <c r="A45" s="41" t="inlineStr">
         <is>
           <t>AI subscriptions</t>
@@ -3363,7 +3363,7 @@
       </c>
       <c r="G45" s="21" t="inlineStr">
         <is>
-          <t>Per HJ item 5. Base links live to the 'AI Subscriptions' tab. Low = trimmed stack; High = full stack plus extra seats as the marketing team scales.</t>
+          <t>Per management (marketing/technology brief, item 5). Base links live to the 'AI Subscriptions' tab. Low = trimmed stack; High = full stack plus extra seats as the marketing team scales.</t>
         </is>
       </c>
     </row>
@@ -4433,7 +4433,7 @@
       </c>
       <c r="F10" s="21" t="inlineStr">
         <is>
-          <t>Per HJ: one unit only. Multiply on the 'Unit Setup' tab for portfolio scale.</t>
+          <t>Per management: one unit only. Multiply on the 'Unit Setup' tab for portfolio scale.</t>
         </is>
       </c>
     </row>
@@ -5127,7 +5127,7 @@
       </c>
       <c r="K15" s="21" t="inlineStr">
         <is>
-          <t>Actual figure supplied by HJ — AED 137.</t>
+          <t>Actual figure supplied by management — AED 137.</t>
         </is>
       </c>
     </row>
@@ -5282,7 +5282,7 @@
       </c>
       <c r="K19" s="21" t="inlineStr">
         <is>
-          <t>Actual figure supplied by HJ — AED 387 for 3 years.</t>
+          <t>Actual figure supplied by management — AED 387 for 3 years.</t>
         </is>
       </c>
     </row>
@@ -5558,7 +5558,7 @@
       </c>
       <c r="K25" s="21" t="inlineStr">
         <is>
-          <t>One-off build of the AI operating layer. The recurring subscription cost sits in OPEX per HJ item 5.</t>
+          <t>One-off build of the AI operating layer. The recurring subscription cost sits in OPEX per management item 5.</t>
         </is>
       </c>
     </row>
@@ -6430,7 +6430,7 @@
       </c>
       <c r="K51" s="36" t="inlineStr">
         <is>
-          <t>Links to 'Unit Setup (1 Unit)'. Per HJ, sized for one unit only.</t>
+          <t>Links to 'Unit Setup (1 Unit)'. Per management, sized for one unit only.</t>
         </is>
       </c>
     </row>
@@ -7073,7 +7073,7 @@
     <row r="21" ht="26" customHeight="1">
       <c r="A21" s="63" t="inlineStr">
         <is>
-          <t>Per HJ, the CAPEX total is built for ONE unit. This table shows what the same unit-setup cost becomes at portfolio scale, against the Business Profile's 70–80 unit Year-1 target.</t>
+          <t>Per management, the CAPEX total is built for ONE unit. This table shows what the same unit-setup cost becomes at portfolio scale, against the Business Profile's 70–80 unit Year-1 target.</t>
         </is>
       </c>
     </row>
@@ -7302,7 +7302,7 @@
       <c r="E5" s="17" t="n"/>
       <c r="F5" s="21" t="inlineStr">
         <is>
-          <t>Understated by design: directors work unpaid per HJ. One ops person for a 70–80 unit portfolio is thin — see the notes below.</t>
+          <t>Understated by design: directors work unpaid per management. One ops person for a 70–80 unit portfolio is thin — see the notes below.</t>
         </is>
       </c>
     </row>
@@ -7402,7 +7402,7 @@
       <c r="E9" s="17" t="n"/>
       <c r="F9" s="21" t="inlineStr">
         <is>
-          <t>Part fixed (AI, Workspace, website), part per-unit (PMS, pricing, locks). Includes HJ item 5.</t>
+          <t>Part fixed (AI, Workspace, website), part per-unit (PMS, pricing, locks). Includes the AI subscriptions specified by management.</t>
         </is>
       </c>
     </row>
@@ -8371,7 +8371,7 @@
       </c>
       <c r="B12" s="70" t="inlineStr">
         <is>
-          <t>Both run M1–M2 per HJ</t>
+          <t>Both run M1–M2 per management</t>
         </is>
       </c>
       <c r="C12" s="77">
@@ -8433,7 +8433,7 @@
       </c>
       <c r="B13" s="70" t="inlineStr">
         <is>
-          <t>Both run M1–M2 per HJ</t>
+          <t>Both run M1–M2 per management</t>
         </is>
       </c>
       <c r="C13" s="77">
@@ -8517,7 +8517,7 @@
       </c>
       <c r="B16" s="70" t="inlineStr">
         <is>
-          <t>Per HJ — nil</t>
+          <t>Per management — nil</t>
         </is>
       </c>
       <c r="C16" s="22">
@@ -8582,7 +8582,7 @@
       </c>
       <c r="B17" s="70" t="inlineStr">
         <is>
-          <t>Per HJ — 1 x AED 3,000</t>
+          <t>Per management — 1 x AED 3,000</t>
         </is>
       </c>
       <c r="C17" s="22">
@@ -9327,7 +9327,7 @@
       </c>
       <c r="B32" s="70" t="inlineStr">
         <is>
-          <t>Per HJ</t>
+          <t>Per management</t>
         </is>
       </c>
       <c r="C32" s="81">
@@ -9392,7 +9392,7 @@
       </c>
       <c r="B33" s="70" t="inlineStr">
         <is>
-          <t>Added by Claude</t>
+          <t>Not in original brief</t>
         </is>
       </c>
       <c r="C33" s="81">
@@ -9457,7 +9457,7 @@
       </c>
       <c r="B34" s="70" t="inlineStr">
         <is>
-          <t>Added by Claude</t>
+          <t>Not in original brief</t>
         </is>
       </c>
       <c r="C34" s="81">
@@ -9583,7 +9583,7 @@
       </c>
       <c r="B36" s="70" t="inlineStr">
         <is>
-          <t>Added by Claude</t>
+          <t>Not in original brief</t>
         </is>
       </c>
       <c r="C36" s="81">
@@ -9707,7 +9707,7 @@
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>D.  UNIT-ACQUISITION COMMISSION  —  the 2% per HJ, ongoing</t>
+          <t>D.  UNIT-ACQUISITION COMMISSION  —  the 2% per management, ongoing</t>
         </is>
       </c>
       <c r="B39" s="5" t="n"/>
@@ -10080,7 +10080,7 @@
       </c>
       <c r="B47" s="70" t="inlineStr">
         <is>
-          <t>Per HJ — see 'AI Subscriptions' tab</t>
+          <t>Per management — see 'AI Subscriptions' tab</t>
         </is>
       </c>
       <c r="C47" s="82">
@@ -12650,7 +12650,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Both options run in parallel for Months 1–2 per HJ. This tab is what you use to pick one.</t>
+          <t>Both options run in parallel for Months 1–2 per management. This tab is what you use to pick one.</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -12926,7 +12926,7 @@
       </c>
       <c r="G14" s="36" t="inlineStr">
         <is>
-          <t>Both at 4 hours per day per HJ.</t>
+          <t>Both at 4 hours per day per management.</t>
         </is>
       </c>
     </row>
@@ -13028,7 +13028,7 @@
       </c>
       <c r="G22" s="36" t="inlineStr">
         <is>
-          <t>The total price of the experiment HJ described.</t>
+          <t>The total price of the experiment specified by management.</t>
         </is>
       </c>
     </row>

</xml_diff>